<commit_message>
EKG-URT-FRM-02 — Devreye Alma Kontrol Listesi (istasyon bazında)
</commit_message>
<xml_diff>
--- a/EKG_Kalite_Yönetim_Sistemi/05_Üretime Başlangıç ve Hata Önleme/01_SP&EP1 - Başlangıç ve İlk Parça/EKG-URT-FRM-02_Devreye Alma Kontrol Listesi (istasyon bazında).xlsx
+++ b/EKG_Kalite_Yönetim_Sistemi/05_Üretime Başlangıç ve Hata Önleme/01_SP&EP1 - Başlangıç ve İlk Parça/EKG-URT-FRM-02_Devreye Alma Kontrol Listesi (istasyon bazında).xlsx
@@ -1037,14 +1037,14 @@
     <row r="41" ht="35" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
+          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19, 49, 53. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="21" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12</t>
+          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12; MRS SP&amp;EPE1 ve SP&amp;EPE3 — başlangıç başarısızlığı, duruş ve hurda kanıtı</t>
         </is>
       </c>
     </row>
@@ -1348,14 +1348,14 @@
     <row r="28" ht="35" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
+          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19, 49, 53. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="21" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12</t>
+          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12; MRS SP&amp;EPE1 ve SP&amp;EPE3 — başlangıç başarısızlığı, duruş ve hurda kanıtı</t>
         </is>
       </c>
     </row>
@@ -1693,14 +1693,14 @@
     <row r="31" ht="35" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
+          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19, 49, 53. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="21" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12</t>
+          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12; MRS SP&amp;EPE1 ve SP&amp;EPE3 — başlangıç başarısızlığı, duruş ve hurda kanıtı</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1916,60 +1916,70 @@
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="n"/>
     </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="16" ht="35" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Başlangıç sapmasına bağlı gerçek duruş başlangıç-bitiş saatleri / duruş dakika / veri kaydı</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+    </row>
+    <row r="17" ht="35" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Başlangıç kaynaklı hurda / ayıklama miktarı, birimi ve ürün karar kaydı</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Etkilenen lot / seri aralığı</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Konum / proses</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Miktar / birim</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Blokaj / ayırma kaydı</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Koruma / inceleme işlemi</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Ürün kararı / yetkili / tarih</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>İlişkili kayıt no</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="n"/>
@@ -2025,81 +2035,79 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
     </row>
-    <row r="27" ht="21" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="9" t="n"/>
+      <c r="B26" s="9" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+    </row>
+    <row r="29" ht="21" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>İstasyon, ayar/deneme parçaları, yarı mamul, sonraki istasyonlar, stok, transit ve gerekiyorsa müşterideki ürünler kapsama alınır. Belirsiz ürünü uygun saymayın.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="21" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="30" ht="21" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Miktar ve konum gerçek kayıtla belirlenir. Ürün kararı ile hat serbest bırakma kararı ayrı izlenir; teknik sınır veya müşteri onayı varsayılmaz.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="34" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Faaliyet no</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Düzeltme / faaliyet</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>Sorumlu</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Termin</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>Tekrar kontrol / ilk parça kaydı</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>Gerçek tekrar sonucu / kanıt</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>Doğrulayan / tarih</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>Durum</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="9" t="n"/>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="9" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="11" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="11" t="n"/>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="11" t="n"/>
-      <c r="G32" s="11" t="n"/>
-      <c r="H32" s="11" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="9" t="n"/>
@@ -2131,82 +2139,114 @@
       <c r="G35" s="9" t="n"/>
       <c r="H35" s="9" t="n"/>
     </row>
-    <row r="37" ht="21" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>İlgili EP fonksiyonu, parametre ve gerekli ilk parça kontrolü uygun sonuçla tekrar doğrulanmadan hat serbest bırakılamaz. Tamamlanmayan kontrol yapılmış gösterilmez.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="21" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>EP by-pass veya alternatif proses bu formda OK işaretlenerek onaylanamaz; EKG-KLT-FRM-42 üzerinden risk, süre/lot sınırı, ek kontrol ve gerekli onaylar izlenir.</t>
-        </is>
-      </c>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="11" t="n"/>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="11" t="n"/>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="9" t="n"/>
+      <c r="B37" s="9" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
     </row>
     <row r="39" ht="21" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Gerekli yeniden başlatma kararı İlk Parça ve Hat Kararı sekmesine aynı kayıt numarasıyla bağlanır.</t>
+          <t>İlgili EP fonksiyonu, parametre ve gerekli ilk parça kontrolü uygun sonuçla tekrar doğrulanmadan hat serbest bırakılamaz. Tamamlanmayan kontrol yapılmış gösterilmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="21" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>EP by-pass veya alternatif proses bu formda OK işaretlenerek onaylanamaz; EKG-KLT-FRM-42 üzerinden risk, süre/lot sınırı, ek kontrol ve gerekli onaylar izlenir.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="21" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Kaynak: MRS #5 PDF s.9–10, 12 ve 17/19. Uygulama bağlantıları: EKG-URT-PRS-02, EKG-KLT-PRS-08, EKG-KLT-FRM-10 ve EKG-KLT-FRM-42.</t>
+          <t>Gerekli yeniden başlatma kararı İlk Parça ve Hat Kararı sekmesine aynı kayıt numarasıyla bağlanır.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="21" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="21" customHeight="1">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12</t>
+          <t>Kaynak: MRS #5 PDF s.9–10, 12 ve 17/19. Uygulama bağlantıları: EKG-URT-PRS-02, EKG-KLT-PRS-08, EKG-KLT-FRM-10 ve EKG-KLT-FRM-42.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="21" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Bu olayın başarısız başlatma, duruş ve hurda bilgileri dönemsel başlangıç etkinliği takibine alınır. Eksik kayıt başarılı kontrol veya sıfır kayıp olarak sayılmaz; EP arızası EKG-KLT-FRM-10 kayıt numarasıyla ayrıştırılır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="35" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Kaynak: Stellantis MRS #5, V1.0, Doc-Info 01601_13_00117; sağlanan PDF s. 8, 9, 10, 11, 12, 13, 15, 16, 17, 18, 19, 49, 53. NSA V8 eşlemesi, kullanıcının paylaştığı belge listesindeki referanstır; MRS kodlarıyla ayrı izlenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="21" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Kriter izleme: SP&amp;EP11; SP&amp;EP12; MRS SP&amp;EPE1 ve SP&amp;EPE3 — başlangıç başarısızlığı, duruş ve hurda kanıtı</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="34">
+    <mergeCell ref="A48:H48"/>
     <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C9:H9"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="C12:H12"/>
+    <mergeCell ref="A45:H45"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="C11:H11"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A41:H41"/>
     <mergeCell ref="C8:H8"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="C17:H17"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="C13:H13"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C15:H15"/>
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A29:H29"/>
     <mergeCell ref="C14:H14"/>
     <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A44:H44"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H31:H35" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Listeden bir değer seçin." type="list">
+    <dataValidation sqref="H33:H37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Listeden bir değer seçin." type="list">
       <formula1>"Açık,Uygulandı,Doğrulandı"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>